<commit_message>
Seed file insertion successfully completed with proper sanity checks
</commit_message>
<xml_diff>
--- a/Master_data.xlsx
+++ b/Master_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dineshreddy/Desktop/ongc_digital_workspace/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01D0886C-A5A8-C547-90F3-3818995C96D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{800FF617-FEBD-604B-86F1-C059A7DD5E64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16260" xr2:uid="{F00B2AF0-4FD8-E844-B457-FFF12CCB774B}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16140" xr2:uid="{F00B2AF0-4FD8-E844-B457-FFF12CCB774B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>